<commit_message>
Add formula to the new report card template, also adjust the report card config on the database, update the classes subjects and curriculums.
</commit_message>
<xml_diff>
--- a/public/files/report_card_templates/Grade 1-3 Matatag.xlsx
+++ b/public/files/report_card_templates/Grade 1-3 Matatag.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\schoolsys\public\files\report_card_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586AEE5B-2B2E-46E3-BB22-719C868325BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB4D0525-354C-4EE8-8618-C95EA710B423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -809,7 +809,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FFC00000"/>
@@ -840,11 +850,6 @@
     <dxf>
       <font>
         <strike val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FFC00000"/>
       </font>
     </dxf>
@@ -1462,24 +1467,36 @@
       <c r="K8" s="36"/>
       <c r="L8" s="36"/>
       <c r="M8" s="36"/>
-      <c r="N8" s="26"/>
+      <c r="N8" s="26" t="str">
+        <f>IF(((N9+N10)/2)&gt;0, (N9+N10)/2, "")</f>
+        <v/>
+      </c>
       <c r="O8" s="26"/>
       <c r="P8" s="26"/>
       <c r="Q8" s="26"/>
-      <c r="R8" s="26"/>
+      <c r="R8" s="26" t="str">
+        <f t="shared" ref="R8" si="0">IF(((R9+R10)/2)&gt;0, (R9+R10)/2, "")</f>
+        <v/>
+      </c>
       <c r="S8" s="26"/>
       <c r="T8" s="26"/>
       <c r="U8" s="26"/>
-      <c r="V8" s="26"/>
+      <c r="V8" s="26" t="str">
+        <f t="shared" ref="V8" si="1">IF(((V9+V10)/2)&gt;0, (V9+V10)/2, "")</f>
+        <v/>
+      </c>
       <c r="W8" s="26"/>
       <c r="X8" s="26"/>
       <c r="Y8" s="26"/>
-      <c r="Z8" s="26"/>
+      <c r="Z8" s="26" t="str">
+        <f t="shared" ref="Z8" si="2">IF(((Z9+Z10)/2)&gt;0, (Z9+Z10)/2, "")</f>
+        <v/>
+      </c>
       <c r="AA8" s="26"/>
       <c r="AB8" s="26"/>
       <c r="AC8" s="26"/>
       <c r="AD8" s="27" t="str">
-        <f t="shared" ref="AD8:AD15" si="0">IF(COUNT(N8:AC8)=4,SUM(N8:AC8)/4,"")</f>
+        <f t="shared" ref="AD8:AD15" si="3">IF(COUNT(N8:AC8)=4,SUM(N8:AC8)/4,"")</f>
         <v/>
       </c>
       <c r="AE8" s="28"/>
@@ -1488,7 +1505,7 @@
       <c r="AH8" s="28"/>
       <c r="AI8" s="29"/>
       <c r="AJ8" s="26" t="str">
-        <f t="shared" ref="AJ8:AJ15" si="1">IF(AD8&lt;&gt;"",IF(AD8 &gt;= 75, "Passed", "Failed"),"")</f>
+        <f t="shared" ref="AJ8:AJ15" si="4">IF(AD8&lt;&gt;"",IF(AD8 &gt;= 75, "Passed", "Failed"),"")</f>
         <v/>
       </c>
       <c r="AK8" s="26"/>
@@ -1529,7 +1546,7 @@
       <c r="AB9" s="26"/>
       <c r="AC9" s="26"/>
       <c r="AD9" s="27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AE9" s="28"/>
@@ -1538,7 +1555,7 @@
       <c r="AH9" s="28"/>
       <c r="AI9" s="29"/>
       <c r="AJ9" s="26" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AK9" s="26"/>
@@ -1562,10 +1579,10 @@
       <c r="K10" s="36"/>
       <c r="L10" s="36"/>
       <c r="M10" s="36"/>
-      <c r="N10" s="26"/>
-      <c r="O10" s="26"/>
-      <c r="P10" s="26"/>
-      <c r="Q10" s="26"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="31"/>
+      <c r="P10" s="31"/>
+      <c r="Q10" s="32"/>
       <c r="R10" s="26"/>
       <c r="S10" s="26"/>
       <c r="T10" s="26"/>
@@ -1579,7 +1596,7 @@
       <c r="AB10" s="26"/>
       <c r="AC10" s="26"/>
       <c r="AD10" s="27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AE10" s="28"/>
@@ -1588,7 +1605,7 @@
       <c r="AH10" s="28"/>
       <c r="AI10" s="29"/>
       <c r="AJ10" s="26" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AK10" s="26"/>
@@ -1629,7 +1646,7 @@
       <c r="AB11" s="26"/>
       <c r="AC11" s="26"/>
       <c r="AD11" s="27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AE11" s="28"/>
@@ -1638,7 +1655,7 @@
       <c r="AH11" s="28"/>
       <c r="AI11" s="29"/>
       <c r="AJ11" s="26" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AK11" s="26"/>
@@ -1662,24 +1679,36 @@
       <c r="K12" s="36"/>
       <c r="L12" s="36"/>
       <c r="M12" s="36"/>
-      <c r="N12" s="26"/>
+      <c r="N12" s="26" t="str">
+        <f>IF((N13*0.6)+(N14*0.2)+(N15*0.2)&gt;0,(N13*0.6)+(N14*0.2)+(N15*0.2), "")</f>
+        <v/>
+      </c>
       <c r="O12" s="26"/>
       <c r="P12" s="26"/>
       <c r="Q12" s="26"/>
-      <c r="R12" s="26"/>
+      <c r="R12" s="26" t="str">
+        <f t="shared" ref="R12" si="5">IF((R13*0.6)+(R14*0.2)+(R15*0.2)&gt;0,(R13*0.6)+(R14*0.2)+(R15*0.2), "")</f>
+        <v/>
+      </c>
       <c r="S12" s="26"/>
       <c r="T12" s="26"/>
       <c r="U12" s="26"/>
-      <c r="V12" s="26"/>
+      <c r="V12" s="26" t="str">
+        <f t="shared" ref="V12" si="6">IF((V13*0.6)+(V14*0.2)+(V15*0.2)&gt;0,(V13*0.6)+(V14*0.2)+(V15*0.2), "")</f>
+        <v/>
+      </c>
       <c r="W12" s="26"/>
       <c r="X12" s="26"/>
       <c r="Y12" s="26"/>
-      <c r="Z12" s="26"/>
+      <c r="Z12" s="26" t="str">
+        <f t="shared" ref="Z12" si="7">IF((Z13*0.6)+(Z14*0.2)+(Z15*0.2)&gt;0,(Z13*0.6)+(Z14*0.2)+(Z15*0.2), "")</f>
+        <v/>
+      </c>
       <c r="AA12" s="26"/>
       <c r="AB12" s="26"/>
       <c r="AC12" s="26"/>
       <c r="AD12" s="27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AE12" s="28"/>
@@ -1688,7 +1717,7 @@
       <c r="AH12" s="28"/>
       <c r="AI12" s="29"/>
       <c r="AJ12" s="26" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AK12" s="26"/>
@@ -1729,7 +1758,7 @@
       <c r="AB13" s="26"/>
       <c r="AC13" s="26"/>
       <c r="AD13" s="27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AE13" s="28"/>
@@ -1738,7 +1767,7 @@
       <c r="AH13" s="28"/>
       <c r="AI13" s="29"/>
       <c r="AJ13" s="26" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AK13" s="26"/>
@@ -1779,7 +1808,7 @@
       <c r="AB14" s="26"/>
       <c r="AC14" s="26"/>
       <c r="AD14" s="27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AE14" s="28"/>
@@ -1788,7 +1817,7 @@
       <c r="AH14" s="28"/>
       <c r="AI14" s="29"/>
       <c r="AJ14" s="26" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AK14" s="26"/>
@@ -1829,7 +1858,7 @@
       <c r="AB15" s="26"/>
       <c r="AC15" s="26"/>
       <c r="AD15" s="27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="AE15" s="28"/>
@@ -1838,7 +1867,7 @@
       <c r="AH15" s="28"/>
       <c r="AI15" s="29"/>
       <c r="AJ15" s="26" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="AK15" s="26"/>
@@ -1862,33 +1891,51 @@
       <c r="K16" s="76"/>
       <c r="L16" s="76"/>
       <c r="M16" s="77"/>
-      <c r="N16" s="26"/>
+      <c r="N16" s="26" t="str">
+        <f>IF((N17*0.6)+(N18*0.2)+(N19*0.2)&gt;0, (N17*0.6)+(N18*0.2)+(N19*0.2), "")</f>
+        <v/>
+      </c>
       <c r="O16" s="26"/>
       <c r="P16" s="26"/>
       <c r="Q16" s="26"/>
-      <c r="R16" s="26"/>
+      <c r="R16" s="26" t="str">
+        <f t="shared" ref="R16" si="8">IF((R17*0.6)+(R18*0.2)+(R19*0.2)&gt;0, (R17*0.6)+(R18*0.2)+(R19*0.2), "")</f>
+        <v/>
+      </c>
       <c r="S16" s="26"/>
       <c r="T16" s="26"/>
       <c r="U16" s="26"/>
-      <c r="V16" s="26"/>
+      <c r="V16" s="26" t="str">
+        <f t="shared" ref="V16" si="9">IF((V17*0.6)+(V18*0.2)+(V19*0.2)&gt;0, (V17*0.6)+(V18*0.2)+(V19*0.2), "")</f>
+        <v/>
+      </c>
       <c r="W16" s="26"/>
       <c r="X16" s="26"/>
       <c r="Y16" s="26"/>
-      <c r="Z16" s="26"/>
+      <c r="Z16" s="26" t="str">
+        <f t="shared" ref="Z16" si="10">IF((Z17*0.6)+(Z18*0.2)+(Z19*0.2)&gt;0, (Z17*0.6)+(Z18*0.2)+(Z19*0.2), "")</f>
+        <v/>
+      </c>
       <c r="AA16" s="26"/>
       <c r="AB16" s="26"/>
       <c r="AC16" s="26"/>
-      <c r="AD16" s="27"/>
+      <c r="AD16" s="27" t="str">
+        <f t="shared" ref="AD16" si="11">IF(COUNT(N16:AC16)=4,SUM(N16:AC16)/4,"")</f>
+        <v/>
+      </c>
       <c r="AE16" s="28"/>
       <c r="AF16" s="28"/>
       <c r="AG16" s="28"/>
       <c r="AH16" s="28"/>
       <c r="AI16" s="29"/>
-      <c r="AJ16" s="30"/>
-      <c r="AK16" s="31"/>
-      <c r="AL16" s="31"/>
-      <c r="AM16" s="31"/>
-      <c r="AN16" s="32"/>
+      <c r="AJ16" s="26" t="str">
+        <f t="shared" ref="AJ16" si="12">IF(AD16&lt;&gt;"",IF(AD16 &gt;= 75, "Passed", "Failed"),"")</f>
+        <v/>
+      </c>
+      <c r="AK16" s="26"/>
+      <c r="AL16" s="26"/>
+      <c r="AM16" s="26"/>
+      <c r="AN16" s="26"/>
     </row>
     <row r="17" spans="1:40" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6"/>
@@ -1923,7 +1970,7 @@
       <c r="AB17" s="26"/>
       <c r="AC17" s="26"/>
       <c r="AD17" s="27" t="str">
-        <f t="shared" ref="AD17:AD19" si="2">IF(COUNT(N17:AC17)=4,SUM(N17:AC17)/4,"")</f>
+        <f t="shared" ref="AD17:AD19" si="13">IF(COUNT(N17:AC17)=4,SUM(N17:AC17)/4,"")</f>
         <v/>
       </c>
       <c r="AE17" s="28"/>
@@ -1932,7 +1979,7 @@
       <c r="AH17" s="28"/>
       <c r="AI17" s="29"/>
       <c r="AJ17" s="26" t="str">
-        <f t="shared" ref="AJ17" si="3">IF(AD17&lt;&gt;"",IF(AD17 &gt;= 75, "Passed", "Failed"),"")</f>
+        <f t="shared" ref="AJ17" si="14">IF(AD17&lt;&gt;"",IF(AD17 &gt;= 75, "Passed", "Failed"),"")</f>
         <v/>
       </c>
       <c r="AK17" s="26"/>
@@ -1973,7 +2020,7 @@
       <c r="AB18" s="26"/>
       <c r="AC18" s="26"/>
       <c r="AD18" s="27" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="AE18" s="28"/>
@@ -1982,7 +2029,7 @@
       <c r="AH18" s="28"/>
       <c r="AI18" s="29"/>
       <c r="AJ18" s="26" t="str">
-        <f t="shared" ref="AJ18:AJ19" si="4">IF(AD18&lt;&gt;"",IF(AD18 &gt;= 75, "Passed", "Failed"),"")</f>
+        <f t="shared" ref="AJ18:AJ19" si="15">IF(AD18&lt;&gt;"",IF(AD18 &gt;= 75, "Passed", "Failed"),"")</f>
         <v/>
       </c>
       <c r="AK18" s="26"/>
@@ -2023,7 +2070,7 @@
       <c r="AB19" s="26"/>
       <c r="AC19" s="26"/>
       <c r="AD19" s="27" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="AE19" s="28"/>
@@ -2032,7 +2079,7 @@
       <c r="AH19" s="28"/>
       <c r="AI19" s="29"/>
       <c r="AJ19" s="26" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
       <c r="AK19" s="26"/>
@@ -2161,7 +2208,7 @@
       <c r="AB22" s="26"/>
       <c r="AC22" s="26"/>
       <c r="AD22" s="27" t="str">
-        <f t="shared" ref="AD22" si="5">IF(COUNT(N22:AC22)=4,SUM(N22:AC22)/4,"")</f>
+        <f t="shared" ref="AD22" si="16">IF(COUNT(N22:AC22)=4,SUM(N22:AC22)/4,"")</f>
         <v/>
       </c>
       <c r="AE22" s="28"/>
@@ -2170,7 +2217,7 @@
       <c r="AH22" s="28"/>
       <c r="AI22" s="29"/>
       <c r="AJ22" s="26" t="str">
-        <f t="shared" ref="AJ22" si="6">IF(AD22&lt;&gt;"",IF(AD22 &gt;= 75, "Passed", "Failed"),"")</f>
+        <f t="shared" ref="AJ22" si="17">IF(AD22&lt;&gt;"",IF(AD22 &gt;= 75, "Passed", "Failed"),"")</f>
         <v/>
       </c>
       <c r="AK22" s="26"/>
@@ -2195,28 +2242,28 @@
       <c r="L23" s="50"/>
       <c r="M23" s="50"/>
       <c r="N23" s="42" t="str">
-        <f>IF(SUM(N7+N8+N9+N10+N11+N12+N18+N19)/8 &gt; 0, SUM(N7+N8+N9+N10+N11+N12+N18+N19)/8, "")</f>
+        <f>IF(COUNT(N7,N8,N11,N12,N16,N22)=6, AVERAGE(N7,N8,N11,N12,N16,N22),"")</f>
         <v/>
       </c>
       <c r="O23" s="42"/>
       <c r="P23" s="42"/>
       <c r="Q23" s="42"/>
       <c r="R23" s="42" t="str">
-        <f t="shared" ref="R23" si="7">IF(SUM(R7+R8+R9+R10+R11+R12+R18+R19)/8 &gt; 0, SUM(R7+R8+R9+R10+R11+R12+R18+R19)/8, "")</f>
+        <f t="shared" ref="R23" si="18">IF(COUNT(R7,R8,R11,R12,R16,R22)=6, AVERAGE(R7,R8,R11,R12,R16,R22),"")</f>
         <v/>
       </c>
       <c r="S23" s="42"/>
       <c r="T23" s="42"/>
       <c r="U23" s="42"/>
       <c r="V23" s="42" t="str">
-        <f t="shared" ref="V23" si="8">IF(SUM(V7+V8+V9+V10+V11+V12+V18+V19)/8 &gt; 0, SUM(V7+V8+V9+V10+V11+V12+V18+V19)/8, "")</f>
+        <f t="shared" ref="V23" si="19">IF(COUNT(V7,V8,V11,V12,V16,V22)=6, AVERAGE(V7,V8,V11,V12,V16,V22),"")</f>
         <v/>
       </c>
       <c r="W23" s="42"/>
       <c r="X23" s="42"/>
       <c r="Y23" s="42"/>
       <c r="Z23" s="42" t="str">
-        <f t="shared" ref="Z23" si="9">IF(SUM(Z7+Z8+Z9+Z10+Z11+Z12+Z18+Z19)/8 &gt; 0, SUM(Z7+Z8+Z9+Z10+Z11+Z12+Z18+Z19)/8, "")</f>
+        <f t="shared" ref="Z23" si="20">IF(COUNT(Z7,Z8,Z11,Z12,Z16,Z22)=6, AVERAGE(Z7,Z8,Z11,Z12,Z16,Z22),"")</f>
         <v/>
       </c>
       <c r="AA23" s="42"/>
@@ -2228,7 +2275,10 @@
       <c r="AG23" s="57"/>
       <c r="AH23" s="57"/>
       <c r="AI23" s="58"/>
-      <c r="AJ23" s="26"/>
+      <c r="AJ23" s="26" t="str">
+        <f>IF(AD24&lt;&gt;"",IF(AD24 &gt;= 75, "Passed", "Failed"),"")</f>
+        <v/>
+      </c>
       <c r="AK23" s="26"/>
       <c r="AL23" s="26"/>
       <c r="AM23" s="26"/>
@@ -2269,7 +2319,7 @@
       <c r="AB24" s="44"/>
       <c r="AC24" s="45"/>
       <c r="AD24" s="53" t="str">
-        <f>IF(SUM(AD7:AI12,AD18:AI19)/8 &gt; 0, SUM(AD7:AI12,AD18:AI19)/8, "")</f>
+        <f>IF(COUNT(AD7,AD8,AD11,AD12,AD16,AD22)=6, AVERAGE(AD7,AD8,AD11,AD12,AD16,AD22), "")</f>
         <v/>
       </c>
       <c r="AE24" s="54"/>
@@ -2893,17 +2943,17 @@
       </c>
       <c r="Q40" s="39"/>
       <c r="R40" s="39">
-        <f t="shared" ref="R40" si="10">SUM(R28:S39)/12</f>
+        <f t="shared" ref="R40" si="21">SUM(R28:S39)/12</f>
         <v>0</v>
       </c>
       <c r="S40" s="39"/>
       <c r="T40" s="39">
-        <f t="shared" ref="T40" si="11">SUM(T28:U39)/12</f>
+        <f t="shared" ref="T40" si="22">SUM(T28:U39)/12</f>
         <v>0</v>
       </c>
       <c r="U40" s="39"/>
       <c r="V40" s="39">
-        <f t="shared" ref="V40" si="12">SUM(V28:W39)/12</f>
+        <f t="shared" ref="V40" si="23">SUM(V28:W39)/12</f>
         <v>0</v>
       </c>
       <c r="W40" s="39"/>
@@ -3296,38 +3346,43 @@
     <mergeCell ref="V17:Y17"/>
   </mergeCells>
   <conditionalFormatting sqref="N7:AC22">
-    <cfRule type="cellIs" dxfId="6" priority="9" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="10" operator="lessThan">
       <formula>75</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AD7:AI15">
-    <cfRule type="cellIs" dxfId="5" priority="10" operator="lessThan">
+  <conditionalFormatting sqref="AD7:AI16">
+    <cfRule type="cellIs" dxfId="7" priority="11" operator="lessThan">
       <formula>75</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD17:AI19">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="lessThan">
       <formula>75</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD22:AI22">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="lessThan">
       <formula>75</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AJ7:AN15">
-    <cfRule type="cellIs" dxfId="2" priority="6" operator="equal">
+  <conditionalFormatting sqref="AJ7:AN16">
+    <cfRule type="cellIs" dxfId="4" priority="7" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ17:AN19">
-    <cfRule type="cellIs" dxfId="1" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AJ22:AN22">
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+  <conditionalFormatting sqref="AJ22:AN23">
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
       <formula>"Failed"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD24:AI24">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <formula>75</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>